<commit_message>
feat: add Codicon file icons and font family settings
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I101" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I104" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I104"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -4773,6 +4773,117 @@
       </c>
       <c r="H101" s="33" t="n"/>
       <c r="I101" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="32" t="inlineStr">
+        <is>
+          <t>F-101</t>
+        </is>
+      </c>
+      <c r="B102" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C102" s="34" t="inlineStr">
+        <is>
+          <t>Sans UI font and monospace code font (editor.fontFamily / workbench.fontFamily)</t>
+        </is>
+      </c>
+      <c r="D102" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E102" s="32" t="n"/>
+      <c r="F102" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G102" s="34" t="inlineStr">
+        <is>
+          <t>Cascadia Mono / Segoe UI by default; no font files are bundled</t>
+        </is>
+      </c>
+      <c r="H102" s="33" t="n"/>
+      <c r="I102" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="32" t="inlineStr">
+        <is>
+          <t>F-102</t>
+        </is>
+      </c>
+      <c r="B103" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C103" s="34" t="inlineStr">
+        <is>
+          <t>Codicon file and folder icons in the Explorer, tabs and Git lists</t>
+        </is>
+      </c>
+      <c r="D103" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E103" s="32" t="n"/>
+      <c r="F103" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G103" s="34" t="inlineStr">
+        <is>
+          <t>Extension icon themes still take over when chosen</t>
+        </is>
+      </c>
+      <c r="H103" s="33" t="n"/>
+      <c r="I103" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="32" t="inlineStr">
+        <is>
+          <t>F-103</t>
+        </is>
+      </c>
+      <c r="B104" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C104" s="34" t="inlineStr">
+        <is>
+          <t>Bundled UI and code fonts (so the look is the same on every PC)</t>
+        </is>
+      </c>
+      <c r="D104" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E104" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F104" s="32" t="n"/>
+      <c r="G104" s="34" t="inlineStr">
+        <is>
+          <t>Needs font files with a licence that allows it, e.g. Inter and JetBrains Mono (OFL)</t>
+        </is>
+      </c>
+      <c r="H104" s="33" t="n"/>
+      <c r="I104" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add built-in snippets for major languages and update documentation
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I104" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I104"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I112" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I112"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -1404,12 +1404,12 @@
       <c r="E6" s="32" t="n"/>
       <c r="F6" s="32" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>App</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>Not offered in the completion popup</t>
+          <t>Prefix + Tab, popup, tab stops, mirrors, choices, variables, transforms; see F-104 to F-110</t>
         </is>
       </c>
       <c r="H6" s="33" t="n"/>
@@ -1858,23 +1858,23 @@
       </c>
       <c r="C19" s="34" t="inlineStr">
         <is>
-          <t>Completions with snippets in the popup</t>
+          <t>Snippets in the completion popup</t>
         </is>
       </c>
       <c r="D19" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E19" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F19" s="32" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
       <c r="G19" s="34" t="inlineStr">
         <is>
-          <t>Completions are plain text today</t>
+          <t>Language-server completions are still plain text (F-110)</t>
         </is>
       </c>
       <c r="H19" s="33" t="n"/>
@@ -4884,6 +4884,294 @@
       </c>
       <c r="H104" s="33" t="n"/>
       <c r="I104" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="32" t="inlineStr">
+        <is>
+          <t>F-104</t>
+        </is>
+      </c>
+      <c r="B105" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C105" s="34" t="inlineStr">
+        <is>
+          <t>Snippet suggestions in the completion popup (editor.snippetSuggestions)</t>
+        </is>
+      </c>
+      <c r="D105" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E105" s="32" t="n"/>
+      <c r="F105" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G105" s="34" t="n"/>
+      <c r="H105" s="33" t="n"/>
+      <c r="I105" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="32" t="inlineStr">
+        <is>
+          <t>F-105</t>
+        </is>
+      </c>
+      <c r="B106" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C106" s="34" t="inlineStr">
+        <is>
+          <t>Snippet choices dropdown (${1|a,b|})</t>
+        </is>
+      </c>
+      <c r="D106" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E106" s="32" t="n"/>
+      <c r="F106" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G106" s="34" t="inlineStr">
+        <is>
+          <t>Arrows then Enter/Tab</t>
+        </is>
+      </c>
+      <c r="H106" s="33" t="n"/>
+      <c r="I106" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="32" t="inlineStr">
+        <is>
+          <t>F-106</t>
+        </is>
+      </c>
+      <c r="B107" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C107" s="34" t="inlineStr">
+        <is>
+          <t>Snippet variables (clipboard, file, line, local date and time, UUID, RANDOM...)</t>
+        </is>
+      </c>
+      <c r="D107" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E107" s="32" t="n"/>
+      <c r="F107" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G107" s="34" t="inlineStr">
+        <is>
+          <t>Unit-tested; all standard variables</t>
+        </is>
+      </c>
+      <c r="H107" s="33" t="n"/>
+      <c r="I107" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="32" t="inlineStr">
+        <is>
+          <t>F-107</t>
+        </is>
+      </c>
+      <c r="B108" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C108" s="34" t="inlineStr">
+        <is>
+          <t>Snippet transforms (${VAR/regex/format/opts})</t>
+        </is>
+      </c>
+      <c r="D108" s="32" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E108" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F108" s="32" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="G108" s="34" t="inlineStr">
+        <is>
+          <t>Worked out once at insertion; not live as you type</t>
+        </is>
+      </c>
+      <c r="H108" s="33" t="n"/>
+      <c r="I108" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="32" t="inlineStr">
+        <is>
+          <t>F-108</t>
+        </is>
+      </c>
+      <c r="B109" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C109" s="34" t="inlineStr">
+        <is>
+          <t>Configure User Snippets (create per-language / global files, reload on save)</t>
+        </is>
+      </c>
+      <c r="D109" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E109" s="32" t="n"/>
+      <c r="F109" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G109" s="34" t="n"/>
+      <c r="H109" s="33" t="n"/>
+      <c r="I109" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="32" t="inlineStr">
+        <is>
+          <t>F-109</t>
+        </is>
+      </c>
+      <c r="B110" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C110" s="34" t="inlineStr">
+        <is>
+          <t>Snippet tab-stop transforms that follow typing</t>
+        </is>
+      </c>
+      <c r="D110" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E110" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F110" s="32" t="n"/>
+      <c r="G110" s="34" t="n"/>
+      <c r="H110" s="33" t="n"/>
+      <c r="I110" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="32" t="inlineStr">
+        <is>
+          <t>F-110</t>
+        </is>
+      </c>
+      <c r="B111" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C111" s="34" t="inlineStr">
+        <is>
+          <t>Expand language-server snippet-format completions</t>
+        </is>
+      </c>
+      <c r="D111" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E111" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F111" s="32" t="n"/>
+      <c r="G111" s="34" t="inlineStr">
+        <is>
+          <t>Servers are told snippets are not supported, so they send plain text</t>
+        </is>
+      </c>
+      <c r="H111" s="33" t="n"/>
+      <c r="I111" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="32" t="inlineStr">
+        <is>
+          <t>F-111</t>
+        </is>
+      </c>
+      <c r="B112" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C112" s="34" t="inlineStr">
+        <is>
+          <t>Built-in snippets for every language (about 290; editor.builtInSnippets)</t>
+        </is>
+      </c>
+      <c r="D112" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E112" s="32" t="n"/>
+      <c r="F112" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G112" s="34" t="inlineStr">
+        <is>
+          <t>Rust, Python, JS/TS/React, HTML, CSS, Go, C/C++, Java, C#, PHP, Ruby, Lua, SQL, shell, YAML, TOML, JSON, Dockerfile, Makefile, Markdown and all-language ones</t>
+        </is>
+      </c>
+      <c r="H112" s="33" t="n"/>
+      <c r="I112" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Emmet, tag auto-completion, and sticky scroll support
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I112" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I112"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I117" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I117"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -1660,21 +1660,25 @@
       </c>
       <c r="C13" s="34" t="inlineStr">
         <is>
-          <t>Emmet</t>
+          <t>Emmet (HTML, JSX, CSS; Tab to expand)</t>
         </is>
       </c>
       <c r="D13" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E13" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F13" s="32" t="n"/>
-      <c r="G13" s="34" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>A practical subset: no filters, no lorem, fewer CSS abbreviations</t>
+        </is>
+      </c>
       <c r="H13" s="33" t="n"/>
       <c r="I13" s="35" t="n">
         <v>46325</v>
@@ -1731,16 +1735,20 @@
       </c>
       <c r="D15" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E15" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F15" s="32" t="n"/>
-      <c r="G15" s="34" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="n"/>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>From folding regions; hidden with word wrap on</t>
+        </is>
+      </c>
       <c r="H15" s="33" t="n"/>
       <c r="I15" s="35" t="n">
         <v>46325</v>
@@ -1759,21 +1767,25 @@
       </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
-          <t>Linked Editing</t>
+          <t>Linked editing (auto rename paired tags)</t>
         </is>
       </c>
       <c r="D16" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E16" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F16" s="32" t="n"/>
-      <c r="G16" s="34" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E16" s="32" t="n"/>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>HTML, XML, JSX; not for other linked ranges a server might offer</t>
+        </is>
+      </c>
       <c r="H16" s="33" t="n"/>
       <c r="I16" s="35" t="n">
         <v>46325</v>
@@ -5172,6 +5184,187 @@
       </c>
       <c r="H112" s="33" t="n"/>
       <c r="I112" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="32" t="inlineStr">
+        <is>
+          <t>F-112</t>
+        </is>
+      </c>
+      <c r="B113" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C113" s="34" t="inlineStr">
+        <is>
+          <t>Auto closing tags (HTML, XML, JSX, TSX)</t>
+        </is>
+      </c>
+      <c r="D113" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E113" s="32" t="n"/>
+      <c r="F113" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G113" s="34" t="inlineStr">
+        <is>
+          <t>Typing &gt; and &lt;/</t>
+        </is>
+      </c>
+      <c r="H113" s="33" t="n"/>
+      <c r="I113" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="32" t="inlineStr">
+        <is>
+          <t>F-113</t>
+        </is>
+      </c>
+      <c r="B114" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C114" s="34" t="inlineStr">
+        <is>
+          <t>Bracket pair colorization</t>
+        </is>
+      </c>
+      <c r="D114" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E114" s="32" t="n"/>
+      <c r="F114" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G114" s="34" t="inlineStr">
+        <is>
+          <t>Skips strings and line comments; block comments can confuse it</t>
+        </is>
+      </c>
+      <c r="H114" s="33" t="n"/>
+      <c r="I114" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="32" t="inlineStr">
+        <is>
+          <t>F-114</t>
+        </is>
+      </c>
+      <c r="B115" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C115" s="34" t="inlineStr">
+        <is>
+          <t>Word-based suggestions without a language server</t>
+        </is>
+      </c>
+      <c r="D115" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E115" s="32" t="n"/>
+      <c r="F115" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G115" s="34" t="n"/>
+      <c r="H115" s="33" t="n"/>
+      <c r="I115" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="32" t="inlineStr">
+        <is>
+          <t>F-115</t>
+        </is>
+      </c>
+      <c r="B116" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C116" s="34" t="inlineStr">
+        <is>
+          <t>Emmet filters, lorem and the rarer CSS abbreviations</t>
+        </is>
+      </c>
+      <c r="D116" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E116" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F116" s="32" t="n"/>
+      <c r="G116" s="34" t="n"/>
+      <c r="H116" s="33" t="n"/>
+      <c r="I116" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="32" t="inlineStr">
+        <is>
+          <t>F-116</t>
+        </is>
+      </c>
+      <c r="B117" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C117" s="34" t="inlineStr">
+        <is>
+          <t>Auto closing tags for Vue / Svelte / PHP files</t>
+        </is>
+      </c>
+      <c r="D117" s="32" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E117" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F117" s="32" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="G117" s="34" t="inlineStr">
+        <is>
+          <t>Works when an extension names the language vue, svelte, astro, handlebars or razor; never tried with one</t>
+        </is>
+      </c>
+      <c r="H117" s="33" t="n"/>
+      <c r="I117" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add CSV table preview, full Markdown preview, and horizontal scrolling
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I117" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I117"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I125" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I125"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -5365,6 +5365,294 @@
       </c>
       <c r="H117" s="33" t="n"/>
       <c r="I117" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="32" t="inlineStr">
+        <is>
+          <t>F-117</t>
+        </is>
+      </c>
+      <c r="B118" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C118" s="34" t="inlineStr">
+        <is>
+          <t>Horizontal scrolling of long lines (wheel, Shift+wheel, caret reveal)</t>
+        </is>
+      </c>
+      <c r="D118" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E118" s="32" t="n"/>
+      <c r="F118" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G118" s="34" t="inlineStr">
+        <is>
+          <t>No horizontal scroll bar is drawn; word wrap on turns it off</t>
+        </is>
+      </c>
+      <c r="H118" s="33" t="n"/>
+      <c r="I118" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="32" t="inlineStr">
+        <is>
+          <t>F-118</t>
+        </is>
+      </c>
+      <c r="B119" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C119" s="34" t="inlineStr">
+        <is>
+          <t>Scrolling the tab strip with the wheel when many tabs are open</t>
+        </is>
+      </c>
+      <c r="D119" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E119" s="32" t="n"/>
+      <c r="F119" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G119" s="34" t="inlineStr">
+        <is>
+          <t>The active tab is brought into view when it changes</t>
+        </is>
+      </c>
+      <c r="H119" s="33" t="n"/>
+      <c r="I119" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="32" t="inlineStr">
+        <is>
+          <t>F-119</t>
+        </is>
+      </c>
+      <c r="B120" s="33" t="inlineStr">
+        <is>
+          <t>Source control</t>
+        </is>
+      </c>
+      <c r="C120" s="34" t="inlineStr">
+        <is>
+          <t>Horizontal scrolling in the side-by-side diff (both columns together)</t>
+        </is>
+      </c>
+      <c r="D120" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E120" s="32" t="n"/>
+      <c r="F120" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G120" s="34" t="inlineStr">
+        <is>
+          <t>Wheel or Shift+wheel; the inline diff is an editor and scrolls like one</t>
+        </is>
+      </c>
+      <c r="H120" s="33" t="n"/>
+      <c r="I120" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="32" t="inlineStr">
+        <is>
+          <t>F-120</t>
+        </is>
+      </c>
+      <c r="B121" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C121" s="34" t="inlineStr">
+        <is>
+          <t>A horizontal scroll bar and dragging to scroll sideways</t>
+        </is>
+      </c>
+      <c r="D121" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E121" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F121" s="32" t="n"/>
+      <c r="G121" s="34" t="n"/>
+      <c r="H121" s="33" t="n"/>
+      <c r="I121" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="32" t="inlineStr">
+        <is>
+          <t>F-121</t>
+        </is>
+      </c>
+      <c r="B122" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C122" s="34" t="inlineStr">
+        <is>
+          <t>Full-page Markdown preview that replaces the source (Ctrl+Shift+V)</t>
+        </is>
+      </c>
+      <c r="D122" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E122" s="32" t="n"/>
+      <c r="F122" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G122" s="34" t="inlineStr">
+        <is>
+          <t>Editing is blocked while it shows</t>
+        </is>
+      </c>
+      <c r="H122" s="33" t="n"/>
+      <c r="I122" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="32" t="inlineStr">
+        <is>
+          <t>F-122</t>
+        </is>
+      </c>
+      <c r="B123" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C123" s="34" t="inlineStr">
+        <is>
+          <t>Markdown preview: headings anchors, raw HTML blocks (e.g. centred images) and task-list checkboxes</t>
+        </is>
+      </c>
+      <c r="D123" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E123" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F123" s="32" t="n"/>
+      <c r="G123" s="34" t="inlineStr">
+        <is>
+          <t>Links to a heading in the same page are not supported; HTML like &lt;p align&gt; shows as text</t>
+        </is>
+      </c>
+      <c r="H123" s="33" t="n"/>
+      <c r="I123" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="32" t="inlineStr">
+        <is>
+          <t>F-123</t>
+        </is>
+      </c>
+      <c r="B124" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C124" s="34" t="inlineStr">
+        <is>
+          <t>CSV / TSV preview as a table (Ctrl+Shift+V)</t>
+        </is>
+      </c>
+      <c r="D124" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E124" s="32" t="n"/>
+      <c r="F124" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G124" s="34" t="inlineStr">
+        <is>
+          <t>Header row, row numbers, guessed delimiter, quoted fields; first 100,000 rows</t>
+        </is>
+      </c>
+      <c r="H124" s="33" t="n"/>
+      <c r="I124" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="32" t="inlineStr">
+        <is>
+          <t>F-124</t>
+        </is>
+      </c>
+      <c r="B125" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C125" s="34" t="inlineStr">
+        <is>
+          <t>CSV preview: sort, filter, edit cells, header-less mode</t>
+        </is>
+      </c>
+      <c r="D125" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E125" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F125" s="32" t="n"/>
+      <c r="G125" s="34" t="n"/>
+      <c r="H125" s="33" t="n"/>
+      <c r="I125" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
perf: optimize per-keystroke editing aids and add benchmarks
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I125" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I125"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I128" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I128"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:I128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -5653,6 +5653,117 @@
       <c r="G125" s="34" t="n"/>
       <c r="H125" s="33" t="n"/>
       <c r="I125" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="32" t="inlineStr">
+        <is>
+          <t>F-125</t>
+        </is>
+      </c>
+      <c r="B126" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C126" s="34" t="inlineStr">
+        <is>
+          <t>Per-keystroke editing aids kept cheap (bracket depths 4.5x faster, word suggestions 2.7x, tag sync skips text, cached sticky lines)</t>
+        </is>
+      </c>
+      <c r="D126" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E126" s="32" t="n"/>
+      <c r="F126" s="32" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="G126" s="34" t="inlineStr">
+        <is>
+          <t>Timings in the README; benchmarks are ignored tests</t>
+        </is>
+      </c>
+      <c r="H126" s="33" t="n"/>
+      <c r="I126" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="32" t="inlineStr">
+        <is>
+          <t>F-126</t>
+        </is>
+      </c>
+      <c r="B127" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C127" s="34" t="inlineStr">
+        <is>
+          <t>Bracket colouring that recomputes only from the edited line</t>
+        </is>
+      </c>
+      <c r="D127" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E127" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F127" s="32" t="n"/>
+      <c r="G127" s="34" t="inlineStr">
+        <is>
+          <t>Today the whole file is re-scanned after each edit (3.6 ms for 25,000 lines)</t>
+        </is>
+      </c>
+      <c r="H127" s="33" t="n"/>
+      <c r="I127" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="32" t="inlineStr">
+        <is>
+          <t>F-127</t>
+        </is>
+      </c>
+      <c r="B128" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C128" s="34" t="inlineStr">
+        <is>
+          <t>Faster CSV parsing for very large files</t>
+        </is>
+      </c>
+      <c r="D128" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E128" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F128" s="32" t="n"/>
+      <c r="G128" s="34" t="inlineStr">
+        <is>
+          <t>About 60 MB/s; done once when the preview opens</t>
+        </is>
+      </c>
+      <c r="H128" s="33" t="n"/>
+      <c r="I128" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
perf: optimize frame rendering, startup times, and add profiler
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I128" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I128"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I136" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I136"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I128"/>
+  <dimension ref="A1:I136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -5764,6 +5764,298 @@
       </c>
       <c r="H128" s="33" t="n"/>
       <c r="I128" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="32" t="inlineStr">
+        <is>
+          <t>F-128</t>
+        </is>
+      </c>
+      <c r="B129" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C129" s="34" t="inlineStr">
+        <is>
+          <t>Mouse cursor follows what is under it (I-beam over text and inputs, hand over clickable things and links, resize arrows)</t>
+        </is>
+      </c>
+      <c r="D129" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E129" s="32" t="n"/>
+      <c r="F129" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G129" s="34" t="inlineStr">
+        <is>
+          <t>Checked with the real Windows cursor; Ctrl over a word in the editor shows a hand</t>
+        </is>
+      </c>
+      <c r="H129" s="33" t="n"/>
+      <c r="I129" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="32" t="inlineStr">
+        <is>
+          <t>F-129</t>
+        </is>
+      </c>
+      <c r="B130" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C130" s="34" t="inlineStr">
+        <is>
+          <t>Minimap rebuilt incrementally on each edit (was the biggest per-frame cost in big files)</t>
+        </is>
+      </c>
+      <c r="D130" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E130" s="32" t="n"/>
+      <c r="F130" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G130" s="34" t="inlineStr">
+        <is>
+          <t>12 ms to 0 ms in a 21,000-line file</t>
+        </is>
+      </c>
+      <c r="H130" s="33" t="n"/>
+      <c r="I130" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="32" t="inlineStr">
+        <is>
+          <t>F-130</t>
+        </is>
+      </c>
+      <c r="B131" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C131" s="34" t="inlineStr">
+        <is>
+          <t>Syntax colours of visible lines cached per frame</t>
+        </is>
+      </c>
+      <c r="D131" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E131" s="32" t="n"/>
+      <c r="F131" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G131" s="34" t="n"/>
+      <c r="H131" s="33" t="n"/>
+      <c r="I131" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="32" t="inlineStr">
+        <is>
+          <t>F-131</t>
+        </is>
+      </c>
+      <c r="B132" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C132" s="34" t="inlineStr">
+        <is>
+          <t>Highlight query compiled once per language</t>
+        </is>
+      </c>
+      <c r="D132" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E132" s="32" t="n"/>
+      <c r="F132" s="32" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="G132" s="34" t="inlineStr">
+        <is>
+          <t>17 ms saved per extra file of a language</t>
+        </is>
+      </c>
+      <c r="H132" s="33" t="n"/>
+      <c r="I132" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="32" t="inlineStr">
+        <is>
+          <t>F-132</t>
+        </is>
+      </c>
+      <c r="B133" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C133" s="34" t="inlineStr">
+        <is>
+          <t>Faster startup: git found on a thread, gpg lookup deferred, background tabs parsed when shown</t>
+        </is>
+      </c>
+      <c r="D133" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E133" s="32" t="n"/>
+      <c r="F133" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G133" s="34" t="inlineStr">
+        <is>
+          <t>About 200 ms less before the first frame</t>
+        </is>
+      </c>
+      <c r="H133" s="33" t="n"/>
+      <c r="I133" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="32" t="inlineStr">
+        <is>
+          <t>F-133</t>
+        </is>
+      </c>
+      <c r="B134" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C134" s="34" t="inlineStr">
+        <is>
+          <t>Profiling aid (FORGE_PROFILE=1)</t>
+        </is>
+      </c>
+      <c r="D134" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E134" s="32" t="n"/>
+      <c r="F134" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G134" s="34" t="inlineStr">
+        <is>
+          <t>Frames per second, time per step, startup phases</t>
+        </is>
+      </c>
+      <c r="H134" s="33" t="n"/>
+      <c r="I134" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="32" t="inlineStr">
+        <is>
+          <t>F-134</t>
+        </is>
+      </c>
+      <c r="B135" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C135" s="34" t="inlineStr">
+        <is>
+          <t>Incremental or deferred syntax reparse for very large files</t>
+        </is>
+      </c>
+      <c r="D135" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E135" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F135" s="32" t="n"/>
+      <c r="G135" s="34" t="inlineStr">
+        <is>
+          <t>4 ms per keystroke at 0.8 MB comes from tree-sitter walking the top-level nodes</t>
+        </is>
+      </c>
+      <c r="H135" s="33" t="n"/>
+      <c r="I135" s="35" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="32" t="inlineStr">
+        <is>
+          <t>F-135</t>
+        </is>
+      </c>
+      <c r="B136" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C136" s="34" t="inlineStr">
+        <is>
+          <t>Faster start of GPUI itself (about 670 ms)</t>
+        </is>
+      </c>
+      <c r="D136" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E136" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F136" s="32" t="n"/>
+      <c r="G136" s="34" t="inlineStr">
+        <is>
+          <t>Outside Forge's own code</t>
+        </is>
+      </c>
+      <c r="H136" s="33" t="n"/>
+      <c r="I136" s="35" t="n">
         <v>46325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update project logo description in documentation
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I136" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I136"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I141" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I141"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="A1:I141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -6057,6 +6057,207 @@
       <c r="H136" s="33" t="n"/>
       <c r="I136" s="35" t="n">
         <v>46325</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="32" t="inlineStr">
+        <is>
+          <t>F-136</t>
+        </is>
+      </c>
+      <c r="B137" s="33" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="C137" s="34" t="inlineStr">
+        <is>
+          <t>Select text in the terminal and copy it</t>
+        </is>
+      </c>
+      <c r="D137" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E137" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F137" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G137" s="34" t="inlineStr">
+        <is>
+          <t>Drag, double-click word, triple-click line; Ctrl+C / Ctrl+Shift+C / right-click copy; checked in the running app</t>
+        </is>
+      </c>
+      <c r="H137" s="33" t="n"/>
+      <c r="I137" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="32" t="inlineStr">
+        <is>
+          <t>F-137</t>
+        </is>
+      </c>
+      <c r="B138" s="33" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="C138" s="34" t="inlineStr">
+        <is>
+          <t>Clickable links in terminal output</t>
+        </is>
+      </c>
+      <c r="D138" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E138" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F138" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G138" s="34" t="inlineStr">
+        <is>
+          <t>URLs open in the browser, existing file paths (with :line:col) open in the editor; underline and hand cursor on hover. URL opening not clicked in testing</t>
+        </is>
+      </c>
+      <c r="H138" s="33" t="n"/>
+      <c r="I138" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="32" t="inlineStr">
+        <is>
+          <t>F-138</t>
+        </is>
+      </c>
+      <c r="B139" s="33" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="C139" s="34" t="inlineStr">
+        <is>
+          <t>Auto-scroll while dragging a selection past the edge; selecting scrollback</t>
+        </is>
+      </c>
+      <c r="D139" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E139" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F139" s="32" t="n"/>
+      <c r="G139" s="34" t="inlineStr">
+        <is>
+          <t>Selection is cleared when the view scrolls</t>
+        </is>
+      </c>
+      <c r="H139" s="33" t="n"/>
+      <c r="I139" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="32" t="inlineStr">
+        <is>
+          <t>F-139</t>
+        </is>
+      </c>
+      <c r="B140" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C140" s="34" t="inlineStr">
+        <is>
+          <t>Welcome page for the empty editor (logo, quick actions, recent folders)</t>
+        </is>
+      </c>
+      <c r="D140" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E140" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F140" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G140" s="34" t="inlineStr">
+        <is>
+          <t>Actions are clickable; checked in the running app</t>
+        </is>
+      </c>
+      <c r="H140" s="33" t="n"/>
+      <c r="I140" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="32" t="inlineStr">
+        <is>
+          <t>F-140</t>
+        </is>
+      </c>
+      <c r="B141" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C141" s="34" t="inlineStr">
+        <is>
+          <t>Activity bar as an icon row with a boxed active icon, overflow menu, logo in the menu bar</t>
+        </is>
+      </c>
+      <c r="D141" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E141" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F141" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G141" s="34" t="inlineStr">
+        <is>
+          <t>Checked in the running app. Icons for Run and Debug, Testing and Remote are not built (no such views)</t>
+        </is>
+      </c>
+      <c r="H141" s="33" t="n"/>
+      <c r="I141" s="35" t="n">
+        <v>46326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add untitled text files, save as, and preview tabs
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I141" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I141"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I144" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I144"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -6257,6 +6257,125 @@
       </c>
       <c r="H141" s="33" t="n"/>
       <c r="I141" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="32" t="inlineStr">
+        <is>
+          <t>F-141</t>
+        </is>
+      </c>
+      <c r="B142" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C142" s="34" t="inlineStr">
+        <is>
+          <t>Preview (replaceable) tabs from a single click in the Explorer</t>
+        </is>
+      </c>
+      <c r="D142" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E142" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F142" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G142" s="34" t="inlineStr">
+        <is>
+          <t>Italic tab; kept on edit or double-click; setting workbench.editor.enablePreview. Checked in the running app</t>
+        </is>
+      </c>
+      <c r="H142" s="33" t="n"/>
+      <c r="I142" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="32" t="inlineStr">
+        <is>
+          <t>F-142</t>
+        </is>
+      </c>
+      <c r="B143" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C143" s="34" t="inlineStr">
+        <is>
+          <t>Preview tabs from Quick Open, search results and Go to Definition</t>
+        </is>
+      </c>
+      <c r="D143" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E143" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F143" s="32" t="n"/>
+      <c r="G143" s="34" t="inlineStr">
+        <is>
+          <t>Only the Explorer opens preview tabs</t>
+        </is>
+      </c>
+      <c r="H143" s="33" t="n"/>
+      <c r="I143" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="32" t="inlineStr">
+        <is>
+          <t>F-143</t>
+        </is>
+      </c>
+      <c r="B144" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C144" s="34" t="inlineStr">
+        <is>
+          <t>Untitled tabs (Ctrl+N) and Save As</t>
+        </is>
+      </c>
+      <c r="D144" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E144" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F144" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G144" s="34" t="inlineStr">
+        <is>
+          <t>System save dialog; tab becomes the file. Checked in the running app. Not built: choosing a language for an untitled tab, restoring untitled tabs after a restart, prompt to save on window close</t>
+        </is>
+      </c>
+      <c r="H144" s="33" t="n"/>
+      <c r="I144" s="35" t="n">
         <v>46326</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add themed title bar support on Windows 11
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I144" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I144"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I145" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I145"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I144"/>
+  <dimension ref="A1:I145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -6376,6 +6376,47 @@
       </c>
       <c r="H144" s="33" t="n"/>
       <c r="I144" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="32" t="inlineStr">
+        <is>
+          <t>F-144</t>
+        </is>
+      </c>
+      <c r="B145" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C145" s="34" t="inlineStr">
+        <is>
+          <t>Title bar coloured from the theme (Windows 11)</t>
+        </is>
+      </c>
+      <c r="D145" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E145" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F145" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G145" s="34" t="inlineStr">
+        <is>
+          <t>DWM caption colour, text, border and dark mode. Checked with the dark and light themes. A custom title bar with the menu inside it is not built</t>
+        </is>
+      </c>
+      <c r="H145" s="33" t="n"/>
+      <c r="I145" s="35" t="n">
         <v>46326</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add responsive custom title bar with search, navigation, and controls
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -6392,7 +6392,7 @@
       </c>
       <c r="C145" s="34" t="inlineStr">
         <is>
-          <t>Title bar coloured from the theme (Windows 11)</t>
+          <t>Responsive custom title bar: menus (fold into ... and a hamburger), back/forward, search box, layout toggles, settings, window buttons</t>
         </is>
       </c>
       <c r="D145" s="32" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="G145" s="34" t="inlineStr">
         <is>
-          <t>DWM caption colour, text, border and dark mode. Checked with the dark and light themes. A custom title bar with the menu inside it is not built</t>
+          <t>Checked in the running app at five widths; layout rules unit-tested. Not built: account and Copilot icons, secondary side bar and Customize Layout, submenus inside the ... menu. macOS and Linux not checked</t>
         </is>
       </c>
       <c r="H145" s="33" t="n"/>

</xml_diff>

<commit_message>
feat: add symbol outline panel and start window maximized
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I145" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I145"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I148" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I148"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -6417,6 +6417,125 @@
       </c>
       <c r="H145" s="33" t="n"/>
       <c r="I145" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="32" t="inlineStr">
+        <is>
+          <t>F-145</t>
+        </is>
+      </c>
+      <c r="B146" s="33" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="C146" s="34" t="inlineStr">
+        <is>
+          <t>Outline view in the Explorer (symbol tree that follows the caret)</t>
+        </is>
+      </c>
+      <c r="D146" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E146" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F146" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G146" s="34" t="inlineStr">
+        <is>
+          <t>LSP symbols, else a text scan (Markdown, Rust, Python, JS/TS, Go...). Checked in the running app; scan unit-tested</t>
+        </is>
+      </c>
+      <c r="H146" s="33" t="n"/>
+      <c r="I146" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="32" t="inlineStr">
+        <is>
+          <t>F-146</t>
+        </is>
+      </c>
+      <c r="B147" s="33" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="C147" s="34" t="inlineStr">
+        <is>
+          <t>Outline: sort and filter options, breadcrumbs from the outline, resizing the section</t>
+        </is>
+      </c>
+      <c r="D147" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E147" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F147" s="32" t="n"/>
+      <c r="G147" s="34" t="inlineStr">
+        <is>
+          <t>The section has a fixed height and shows symbols in file order</t>
+        </is>
+      </c>
+      <c r="H147" s="33" t="n"/>
+      <c r="I147" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="32" t="inlineStr">
+        <is>
+          <t>F-147</t>
+        </is>
+      </c>
+      <c r="B148" s="33" t="inlineStr">
+        <is>
+          <t>Workbench</t>
+        </is>
+      </c>
+      <c r="C148" s="34" t="inlineStr">
+        <is>
+          <t>Window always opens maximized</t>
+        </is>
+      </c>
+      <c r="D148" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E148" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F148" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G148" s="34" t="inlineStr">
+        <is>
+          <t>Checked in the running app. True full screen (F11, no taskbar) is not built</t>
+        </is>
+      </c>
+      <c r="H148" s="33" t="n"/>
+      <c r="I148" s="35" t="n">
         <v>46326</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add language mode picker, auto-detection, and smart comments
</commit_message>
<xml_diff>
--- a/docs/FEATURES.xlsx
+++ b/docs/FEATURES.xlsx
@@ -422,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I148" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I148"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Features" displayName="Features" ref="A1:I151" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I151"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.00390625" customWidth="1" style="31" min="1" max="1"/>
@@ -6536,6 +6536,125 @@
       </c>
       <c r="H148" s="33" t="n"/>
       <c r="I148" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="32" t="inlineStr">
+        <is>
+          <t>F-148</t>
+        </is>
+      </c>
+      <c r="B149" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C149" s="34" t="inlineStr">
+        <is>
+          <t>Language mode picker (status bar) with Auto Detect, and content-based detection</t>
+        </is>
+      </c>
+      <c r="D149" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E149" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F149" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G149" s="34" t="inlineStr">
+        <is>
+          <t>Name, then shebang/markup/shape of the code; embedded languages follow. Checked in the running app; detection unit-tested</t>
+        </is>
+      </c>
+      <c r="H149" s="33" t="n"/>
+      <c r="I149" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="32" t="inlineStr">
+        <is>
+          <t>F-149</t>
+        </is>
+      </c>
+      <c r="B150" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C150" s="34" t="inlineStr">
+        <is>
+          <t>Language mode: associate a file extension with a language, languages from extensions in the picker, remember the choice per file</t>
+        </is>
+      </c>
+      <c r="D150" s="32" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E150" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F150" s="32" t="n"/>
+      <c r="G150" s="34" t="inlineStr">
+        <is>
+          <t>A manual choice lasts only while the file is open</t>
+        </is>
+      </c>
+      <c r="H150" s="33" t="n"/>
+      <c r="I150" s="35" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="32" t="inlineStr">
+        <is>
+          <t>F-150</t>
+        </is>
+      </c>
+      <c r="B151" s="33" t="inlineStr">
+        <is>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="C151" s="34" t="inlineStr">
+        <is>
+          <t>Toggle comment works in HTML, CSS, Markdown, XML, JSON and embedded code</t>
+        </is>
+      </c>
+      <c r="D151" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E151" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F151" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G151" s="34" t="inlineStr">
+        <is>
+          <t>HTML, XML, Markdown, CSS: one block comment around the selection (like VS Code's block fallback); line-comment languages: one token per line. Language taken at the caret. Checked in the running app; unit-tested</t>
+        </is>
+      </c>
+      <c r="H151" s="33" t="n"/>
+      <c r="I151" s="35" t="n">
         <v>46326</v>
       </c>
     </row>

</xml_diff>